<commit_message>
Rebuild the pages with the approach note and the new tab
</commit_message>
<xml_diff>
--- a/deliverables/backlog.xlsx
+++ b/deliverables/backlog.xlsx
@@ -2042,7 +2042,7 @@
       <c r="J17" s="2" t="inlineStr">
         <is>
           <t>• Concentrix: named in 7 reviews since 2023, 57% 1–2★ (Long routes / bad clubbing, Helpdesk unhelpful / complaints ignored, Driver behaviour or driving).
-• Wipro: named in 5 reviews since 2023, 60% 1–2★ (Slow to load / hangs, Cab location wrong or lagging, Can't call or message driver).
+• Wipro: named in 5 reviews since 2023, 60% 1–2★ (Can't call or message driver, Slow to load / hangs, Cab location wrong or lagging).
 • HCL: named in 4 reviews since 2023, 75% 1–2★ (Pickup time unpredictable / changed late, Can't see my bookings / trip details, Crash, blank screen or won't open).
 • Tech Mahindra: named in 4 reviews since 2023, 50% 1–2★ (Helpdesk unhelpful / complaints ignored, Long routes / bad clubbing).
 • JPMorgan Chase: named in 3 reviews since 2023, 33% 1–2★ (no specific issue).
@@ -3770,7 +3770,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Evidence: Google Play reviews up to 11 Oct 2026; generated 13 Oct 2026, 01:54.</t>
+          <t>Evidence: Google Play reviews up to 11 Oct 2026; generated 13 Oct 2026, 02:40.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild the pages with India-time stamps
</commit_message>
<xml_diff>
--- a/deliverables/backlog.xlsx
+++ b/deliverables/backlog.xlsx
@@ -2041,9 +2041,9 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>• Concentrix: named in 7 reviews since 2023, 57% 1–2★ (Long routes / bad clubbing, Helpdesk unhelpful / complaints ignored, Driver behaviour or driving).
+          <t>• Concentrix: named in 7 reviews since 2023, 57% 1–2★ (Long routes / bad clubbing, Driver behaviour or driving, Helpdesk unhelpful / complaints ignored).
 • Wipro: named in 5 reviews since 2023, 60% 1–2★ (Can't call or message driver, Slow to load / hangs, Cab location wrong or lagging).
-• HCL: named in 4 reviews since 2023, 75% 1–2★ (Pickup time unpredictable / changed late, Can't see my bookings / trip details, Crash, blank screen or won't open).
+• HCL: named in 4 reviews since 2023, 75% 1–2★ (Can't see my bookings / trip details, Pickup time unpredictable / changed late, Frequent logout / re-login).
 • Tech Mahindra: named in 4 reviews since 2023, 50% 1–2★ (Helpdesk unhelpful / complaints ignored, Long routes / bad clubbing).
 • JPMorgan Chase: named in 3 reviews since 2023, 33% 1–2★ (no specific issue).
 • Small numbers: a lead for the account team, not a verdict.
@@ -3770,7 +3770,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Evidence: Google Play reviews up to 11 Oct 2026; generated 13 Oct 2026, 02:40.</t>
+          <t>Evidence: Google Play reviews up to 11 Oct 2026; generated 13 Oct 2026, 03:30 IST.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild the pages and METHOD.md from today's data
</commit_message>
<xml_diff>
--- a/deliverables/backlog.xlsx
+++ b/deliverables/backlog.xlsx
@@ -615,7 +615,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>MoveInSync stopped replying to Play Store reviews. Unhappy employees hear nothing back, and every new employee reading the store page sees complaints left unanswered, while the closest comparison app answers its negative reviews.</t>
+          <t>Unanswered reviews: unhappy employees hear nothing back, and every new employee reading the store page sees the complaints left unanswered. The evidence gives the current reply rates for MoveInSync and the closest comparison app.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Triage the crash rise in 12.19.0 with Android vitals and decide hotfix vs. rollback</t>
+          <t>Triage crashes in release 12.19.0 with Android vitals and decide hotfix vs. rollback</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>"Crash, blank screen or won't open" costs the rating more than any other issue and is rising in the latest reviews, led by the newest release. Play may also reduce the app's visibility and show a store-listing warning when crash or ANR rates pass its bad-behaviour thresholds.</t>
+          <t>Crashes, blank screens and an app that won't open; the evidence gives the issue's current rating-cost rank, trend and the latest release's figures. Play may also reduce the app's visibility and show a store-listing warning when crash or ANR rates pass its bad-behaviour thresholds.</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>Stops the current rise; the lasting fix is MIS-05.</t>
+          <t>Contains crashes in the current release; the lasting fix is MIS-05.</t>
         </is>
       </c>
       <c r="Q3" s="2" t="n"/>
@@ -794,7 +794,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Releases ship often, and many reviews calling the app hard to use blame a recent update. A bad release reaches every employee before anyone notices.</t>
+          <t>Releases ship often, and reviews calling the app hard to use blame recent updates. A bad release reaches every employee before anyone notices.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -885,7 +885,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Employees who installed from Google Play are told every few days that the app "was not downloaded from Play Store" and must reinstall. This is rising. The pattern (works, then fails days later) points to an integrity check that fails closed on transient errors or stale verdicts, not to sideloading.</t>
+          <t>Employees who installed from Google Play are told every few days that the app "was not downloaded from Play Store" and must reinstall. The pattern (works, then fails days later) points to an integrity check that fails closed on transient errors or stale verdicts, not to sideloading.</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>Targets the largest single rating cost.</t>
+          <t>Targets the issue's rating cost (its current rank is in the evidence).</t>
         </is>
       </c>
       <c r="Q6" s="3" t="n">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>The redesigned app is called hard to use, often blaming a recent update. The newest named complaint is the seat-belt confirmation that now pops up before the boarding OTP, adding a step and hiding the OTP while the driver waits.</t>
+          <t>The redesigned app is called hard to use, some reviews blaming a recent update. One named complaint is the seat-belt confirmation that now pops up before the boarding OTP, adding a step and hiding the OTP while the driver waits.</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Most ratings come from employees who never write a review, and they rate the app highly. Asking them on Play at a good moment is the cheapest way to add recent positive ratings. The app's own post-trip rating pop-up, by contrast, is itself a complaint. (If the app already calls the In-App Review API, this ticket becomes tuning when it fires.)</t>
+          <t>Employees who rate without writing a review count in the store rating but never appear in reviews; the evidence gives their share and average stars. Asking them on Play at a good moment is the cheapest way to add recent positive ratings. The app's own post-trip rating pop-up, by contrast, is itself a complaint. (If the app already calls the In-App Review API, this ticket becomes tuning when it fires.)</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1380,7 +1380,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Complaints about missing, late or repeated notifications (cab allocated, cab arriving) are emerging in the last 30 days.</t>
+          <t>Complaints about missing, late or repeated notifications (cab allocated, cab arriving); the evidence gives their current share and trend.</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>Early action on an emerging complaint while it is still small.</t>
+          <t>Fixes the cause before the complaint grows.</t>
         </is>
       </c>
       <c r="Q10" s="3" t="n">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Safety concerns are rare in reviews but each one needs action; more reviews praise safety than raise a concern, so safety is a strength to protect.</t>
+          <t>Each safety concern raised in a review needs action, however few there are. The evidence gives the current count, and how many reviews praise safety.</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1692,7 +1692,7 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>Protects a strength; prevents a single incident review from going unanswered.</t>
+          <t>No safety concern raised in a review goes unanswered.</t>
         </is>
       </c>
       <c r="Q13" s="3" t="n">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Share, 12 months</t>
+          <t>Share, last 365d</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
@@ -3770,7 +3770,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Evidence: Google Play reviews up to 11 Oct 2026; generated 13 Oct 2026, 03:30 IST.</t>
+          <t>Evidence: Google Play reviews up to 11 Oct 2026; generated 13 Oct 2026, 03:52 IST.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild METHOD.md with the spot-check
</commit_message>
<xml_diff>
--- a/deliverables/backlog.xlsx
+++ b/deliverables/backlog.xlsx
@@ -2041,9 +2041,9 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>• Concentrix: named in 7 reviews since 2023, 57% 1–2★ (Long routes / bad clubbing, Driver behaviour or driving, Helpdesk unhelpful / complaints ignored).
-• Wipro: named in 5 reviews since 2023, 60% 1–2★ (Can't call or message driver, Slow to load / hangs, Cab location wrong or lagging).
-• HCL: named in 4 reviews since 2023, 75% 1–2★ (Can't see my bookings / trip details, Pickup time unpredictable / changed late, Frequent logout / re-login).
+          <t>• Concentrix: named in 7 reviews since 2023, 57% 1–2★ (Long routes / bad clubbing, Helpdesk unhelpful / complaints ignored, Driver behaviour or driving).
+• Wipro: named in 5 reviews since 2023, 60% 1–2★ (Cab location wrong or lagging, Slow to load / hangs, Can't call or message driver).
+• HCL: named in 4 reviews since 2023, 75% 1–2★ (Pickup time unpredictable / changed late, Can't see my bookings / trip details, Crash, blank screen or won't open).
 • Tech Mahindra: named in 4 reviews since 2023, 50% 1–2★ (Helpdesk unhelpful / complaints ignored, Long routes / bad clubbing).
 • JPMorgan Chase: named in 3 reviews since 2023, 33% 1–2★ (no specific issue).
 • Small numbers: a lead for the account team, not a verdict.
@@ -3770,7 +3770,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Evidence: Google Play reviews up to 11 Oct 2026; generated 13 Oct 2026, 03:52 IST.</t>
+          <t>Evidence: Google Play reviews up to 11 Oct 2026; generated 13 Oct 2026, 04:17 IST.</t>
         </is>
       </c>
     </row>

</xml_diff>